<commit_message>
Adição dos itens 10 e 11
</commit_message>
<xml_diff>
--- a/resultados_cenarios.xlsx
+++ b/resultados_cenarios.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>Cenário</t>
   </si>
@@ -68,6 +68,12 @@
   </si>
   <si>
     <t>Sinal + Estatísticas Globais, Antes e Depois</t>
+  </si>
+  <si>
+    <t>Estatísticas Pre-R</t>
+  </si>
+  <si>
+    <t>Estatísticas Pos-R</t>
   </si>
 </sst>
 </file>
@@ -469,7 +475,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="7" width="13.576428571428572" customWidth="1" bestFit="1"/>
@@ -773,6 +779,64 @@
         <v>0.7834192105799677</v>
       </c>
     </row>
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
+      <c r="A11" s="4">
+        <v>10</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="6">
+        <v>0.9076770818605966</v>
+      </c>
+      <c r="D11" s="6">
+        <v>0.08897078178468018</v>
+      </c>
+      <c r="E11" s="6">
+        <v>0.9881725717539274</v>
+      </c>
+      <c r="F11" s="6">
+        <v>0.4251572327044025</v>
+      </c>
+      <c r="G11" s="6">
+        <v>0.1471484545058772</v>
+      </c>
+      <c r="H11" s="6">
+        <v>0.1624394578746495</v>
+      </c>
+      <c r="I11" s="6">
+        <v>0.5524138191270972</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
+      <c r="A12" s="4">
+        <v>11</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="6">
+        <v>0.888684669400066</v>
+      </c>
+      <c r="D12" s="6">
+        <v>0.2140036851803106</v>
+      </c>
+      <c r="E12" s="6">
+        <v>0.9550195398431637</v>
+      </c>
+      <c r="F12" s="6">
+        <v>0.3186985495883967</v>
+      </c>
+      <c r="G12" s="6">
+        <v>0.2560629921259843</v>
+      </c>
+      <c r="H12" s="6">
+        <v>0.2030126283219027</v>
+      </c>
+      <c r="I12" s="6">
+        <v>0.6700858278334929</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>